<commit_message>
fix: fixed the admin controls over student
</commit_message>
<xml_diff>
--- a/client/public/Student_Import_Template.xlsx
+++ b/client/public/Student_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\archi\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2AC463-6C74-4F55-AEFC-D59F02D822F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFB836B-9BDB-4FF6-89F1-9A0BB47A7E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E2D51B8-E79F-435B-B073-150BC562E547}"/>
   </bookViews>
@@ -568,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -580,21 +580,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1061,39 +1059,39 @@
     <col min="11" max="16384" width="13.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="6" customFormat="1" ht="27.6" thickBot="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:10" s="5" customFormat="1" ht="27.6" thickBot="1">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="27.6" thickBot="1">
+    <row r="2" spans="1:10" ht="15" thickBot="1">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1115,7 +1113,7 @@
       <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" t="s">
         <v>18</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -1125,7 +1123,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="27.6" thickBot="1">
+    <row r="3" spans="1:10" ht="15" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1147,7 +1145,7 @@
       <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" t="s">
         <v>18</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -1157,7 +1155,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="27.6" thickBot="1">
+    <row r="4" spans="1:10" ht="15" thickBot="1">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1179,7 +1177,7 @@
       <c r="G4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -1189,7 +1187,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="27.6" thickBot="1">
+    <row r="5" spans="1:10" ht="15" thickBot="1">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -1211,7 +1209,7 @@
       <c r="G5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" t="s">
         <v>18</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -1222,13 +1220,13 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="27.6" thickBot="1">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-    </row>
-    <row r="15" spans="1:10" ht="28.2" thickBot="1">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" thickBot="1">
       <c r="A15" s="4" t="s">
         <v>34</v>
       </c>
@@ -1243,160 +1241,150 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="28.2" thickBot="1">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="11"/>
-    </row>
-    <row r="17" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A17" s="7" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A17" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="11"/>
-    </row>
-    <row r="18" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A18" s="7" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="11"/>
-    </row>
-    <row r="19" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A19" s="7" t="s">
+    </row>
+    <row r="19" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A19" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="11"/>
-    </row>
-    <row r="20" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A20" s="7" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="11"/>
-    </row>
-    <row r="21" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A21" s="7" t="s">
+    </row>
+    <row r="21" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A21" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E21" s="11"/>
-    </row>
-    <row r="22" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A22" s="7" t="s">
+    </row>
+    <row r="22" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A22" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E22" s="11"/>
-    </row>
-    <row r="23" spans="1:5" ht="42" thickBot="1">
-      <c r="A23" s="7" t="s">
+    </row>
+    <row r="23" spans="1:4" ht="42" thickBot="1">
+      <c r="A23" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E23" s="11"/>
-    </row>
-    <row r="24" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A24" s="7" t="s">
+    </row>
+    <row r="24" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A24" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A25" s="7" t="s">
+    </row>
+    <row r="25" spans="1:4" ht="28.2" thickBot="1">
+      <c r="A25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="11"/>
-    </row>
-    <row r="27" spans="1:5" ht="29.4">
-      <c r="A27" s="8" t="s">
+    </row>
+    <row r="27" spans="1:4" ht="29.4">
+      <c r="A27" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>